<commit_message>
user ticket modules and services
</commit_message>
<xml_diff>
--- a/public/admin/files/questionupload.xlsx
+++ b/public/admin/files/questionupload.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
   <si>
     <t>question</t>
   </si>
@@ -49,6 +49,12 @@
   </si>
   <si>
     <t>No</t>
+  </si>
+  <si>
+    <t>rationale</t>
+  </si>
+  <si>
+    <t>this is a rationale justification</t>
   </si>
 </sst>
 </file>
@@ -387,10 +393,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -409,8 +415,11 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
+      <c r="G1" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -428,6 +437,9 @@
       </c>
       <c r="F2" t="s">
         <v>1</v>
+      </c>
+      <c r="G2" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>